<commit_message>
Add robustness diagnostics and correct attention check key
Corrects attention check response key (ac_2: 5→1, ac_3: 5→1) and implements comprehensive robustness framework. Adds pre-specified alternative CFA models (3-factor and 1-factor competence), validates attention key against observed data, uses theoretical mean (3) for quadrant cuts, and creates decision register documenting methodological decisions. Extends playground with recalculated attention checks and guidance page explaining sample roles and sensitivity workflow. Updates all CFA reporting to include analysis role, sample role, and attention-key status.
</commit_message>
<xml_diff>
--- a/outputs/tables/descriptive_statistics_all_variables.xlsx
+++ b/outputs/tables/descriptive_statistics_all_variables.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
   <si>
     <t xml:space="preserve">variable</t>
   </si>
@@ -369,28 +369,43 @@
     <t xml:space="preserve">minimum_correct_attention_checks</t>
   </si>
   <si>
+    <t xml:space="preserve">sample_role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attention_key_status</t>
+  </si>
+  <si>
     <t xml:space="preserve">all_core</t>
   </si>
   <si>
     <t xml:space="preserve">All core-eligible observations</t>
   </si>
   <si>
+    <t xml:space="preserve">Primary analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validated against observed response coding</t>
+  </si>
+  <si>
     <t xml:space="preserve">fail_at_most_2</t>
   </si>
   <si>
-    <t xml:space="preserve">Failed at most two attention checks</t>
+    <t xml:space="preserve">At least two checks correct (provisional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensitivity analysis; key not yet validated</t>
   </si>
   <si>
     <t xml:space="preserve">fail_at_most_1</t>
   </si>
   <si>
-    <t xml:space="preserve">Failed at most one attention check</t>
+    <t xml:space="preserve">At least three checks correct (provisional)</t>
   </si>
   <si>
     <t xml:space="preserve">pass_all_4</t>
   </si>
   <si>
-    <t xml:space="preserve">Passed all four attention checks</t>
+    <t xml:space="preserve">All four checks correct (provisional)</t>
   </si>
   <si>
     <t xml:space="preserve">model</t>
@@ -611,13 +626,15 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table8" displayName="Table8" ref="A1:D5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:D5"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table8" displayName="Table8" ref="A1:F5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F5"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="sample_key"/>
     <tableColumn id="2" name="sample_label"/>
     <tableColumn id="3" name="minimum_correct_attention_checks"/>
-    <tableColumn id="4" name="n"/>
+    <tableColumn id="4" name="sample_role"/>
+    <tableColumn id="5" name="attention_key_status"/>
+    <tableColumn id="6" name="n"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1856,34 +1873,34 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.815028901734104</v>
+        <v>1.67630057803468</v>
       </c>
       <c r="F7" t="n">
-        <v>0.388434529182873</v>
+        <v>0.654993424097705</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>-1.62070433297123</v>
+        <v>-1.78909452195644</v>
       </c>
       <c r="M7" t="n">
-        <v>0.627202501146863</v>
+        <v>1.67515602756819</v>
       </c>
       <c r="N7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1944,34 +1961,34 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.777043765483072</v>
+        <v>1.61767134599505</v>
       </c>
       <c r="F9" t="n">
-        <v>0.416401166113702</v>
+        <v>0.679074378036414</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>-1.32955916211913</v>
+        <v>-1.50655833137627</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.232462348329883</v>
+        <v>0.797788441478528</v>
       </c>
       <c r="N9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1988,34 +2005,34 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>2.40792733278282</v>
+        <v>0.706028075970273</v>
       </c>
       <c r="F10" t="n">
-        <v>0.705634874799491</v>
+        <v>1.23761500677562</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>4</v>
       </c>
       <c r="L10" t="n">
-        <v>1.42070137834941</v>
+        <v>1.69943319195659</v>
       </c>
       <c r="M10" t="n">
-        <v>0.47253121174125</v>
+        <v>1.61490688820899</v>
       </c>
       <c r="N10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -2076,34 +2093,34 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>1.59207266721718</v>
+        <v>3.29397192402973</v>
       </c>
       <c r="F12" t="n">
-        <v>0.705634874799491</v>
+        <v>1.23761500677562</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>-1.42070137834941</v>
+        <v>-1.69943319195659</v>
       </c>
       <c r="M12" t="n">
-        <v>0.472531211741248</v>
+        <v>1.61490688820899</v>
       </c>
       <c r="N12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -6750,9 +6767,11 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="35.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="43.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="32.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="4.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="43.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="42.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="4.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6766,63 +6785,93 @@
         <v>115</v>
       </c>
       <c r="D1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F2" t="n">
         <v>1211</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="n">
-        <v>872</v>
+      <c r="D3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1073</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
+      <c r="D4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" t="n">
+        <v>980</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
+      <c r="D5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" t="n">
+        <v>823</v>
       </c>
     </row>
   </sheetData>
@@ -6849,30 +6898,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C2" t="n">
         <v>1211</v>
@@ -6884,15 +6933,15 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C3" t="n">
         <v>1211</v>
@@ -6904,15 +6953,15 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C4" t="n">
         <v>1211</v>
@@ -6924,7 +6973,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -6950,24 +6999,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E1" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B2" t="n">
         <v>1211</v>
@@ -6984,7 +7033,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B3" t="n">
         <v>1211</v>
@@ -7001,7 +7050,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B4" t="n">
         <v>1211</v>
@@ -7018,7 +7067,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B5" t="n">
         <v>1211</v>
@@ -7035,7 +7084,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B6" t="n">
         <v>1211</v>
@@ -7052,7 +7101,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B7" t="n">
         <v>1211</v>
@@ -7069,7 +7118,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B8" t="n">
         <v>1211</v>
@@ -7086,7 +7135,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B9" t="n">
         <v>1211</v>

</xml_diff>